<commit_message>
Redesign Bay Frontend Display
</commit_message>
<xml_diff>
--- a/.files/1_Report.xlsx
+++ b/.files/1_Report.xlsx
@@ -8,7 +8,8 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="1 (Copy)" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Summary" sheetId="3" state="visible" r:id="rId3"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -335,6 +336,36 @@
 <wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
   <oneCellAnchor>
     <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="3429000" cy="2571750"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="1" name="Image 1" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId1"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+</wsDr>
+</file>
+
+<file path=xl/drawings/drawing3.xml><?xml version="1.0" encoding="utf-8"?>
+<wsDr xmlns="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing">
+  <oneCellAnchor>
+    <from>
       <col>6</col>
       <colOff>0</colOff>
       <row>39</row>
@@ -654,6 +685,998 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="26" customWidth="1" min="1" max="1"/>
+    <col width="39" customWidth="1" min="2" max="2"/>
+    <col width="2" customWidth="1" min="3" max="3"/>
+    <col width="2" customWidth="1" min="4" max="4"/>
+    <col width="99" customWidth="1" min="5" max="5"/>
+    <col width="13" customWidth="1" min="6" max="6"/>
+    <col width="64" customWidth="1" min="7" max="7"/>
+    <col width="17" customWidth="1" min="8" max="8"/>
+    <col width="28" customWidth="1" min="9" max="9"/>
+    <col width="2" customWidth="1" min="10" max="10"/>
+    <col width="2" customWidth="1" min="11" max="11"/>
+  </cols>
+  <sheetData>
+    <row r="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>System Input</t>
+        </is>
+      </c>
+      <c r="B1" s="2" t="inlineStr">
+        <is>
+          <t>YES 45TU FRONT SET(OG)</t>
+        </is>
+      </c>
+      <c r="E1" s="3" t="inlineStr">
+        <is>
+          <t>PROFILES</t>
+        </is>
+      </c>
+    </row>
+    <row r="2">
+      <c r="A2" s="1" t="inlineStr">
+        <is>
+          <t>Finish</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="inlineStr">
+        <is>
+          <t>Clear</t>
+        </is>
+      </c>
+      <c r="E2" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F2" s="4" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G2" s="4" t="inlineStr">
+        <is>
+          <t>Total Quantity Required</t>
+        </is>
+      </c>
+      <c r="H2" s="4" t="inlineStr">
+        <is>
+          <t>Total List Cost</t>
+        </is>
+      </c>
+      <c r="I2" s="4" t="inlineStr">
+        <is>
+          <t>Discounted Total List Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="3">
+      <c r="A3" s="1" t="inlineStr">
+        <is>
+          <t>Elevation Type</t>
+        </is>
+      </c>
+      <c r="B3" s="2" t="inlineStr">
+        <is>
+          <t>1</t>
+        </is>
+      </c>
+      <c r="E3" t="inlineStr">
+        <is>
+          <t>Vertical Sill/Jamb Screw Spline Assembly (Jamb) / Horizontal Sill/Jamb Screw Spline Assembly (Sill)</t>
+        </is>
+      </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>BE9-2513</t>
+        </is>
+      </c>
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>8ft, 8ft, 0.08ft, 3.97ft, 3.97ft, 3.97ft</t>
+        </is>
+      </c>
+      <c r="H3" s="5" t="n">
+        <v>838</v>
+      </c>
+      <c r="I3" s="5" t="n">
+        <v>514.532</v>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="1" t="inlineStr">
+        <is>
+          <t>Total Count</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="n">
+        <v>1</v>
+      </c>
+      <c r="E4" t="inlineStr">
+        <is>
+          <t>Vertical Flush Filler</t>
+        </is>
+      </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>E9-2512</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>8ft x 3</t>
+        </is>
+      </c>
+      <c r="H4" s="5" t="n">
+        <v>150</v>
+      </c>
+      <c r="I4" s="5" t="n">
+        <v>92.09999999999999</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="1" t="inlineStr">
+        <is>
+          <t>Bays Wide</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="n">
+        <v>4</v>
+      </c>
+      <c r="E5" t="inlineStr">
+        <is>
+          <t>Vertical Two Piece Mullion Screw Spline Assembly</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>BE9-2511</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>8ft x 3</t>
+        </is>
+      </c>
+      <c r="H5" s="5" t="n">
+        <v>497</v>
+      </c>
+      <c r="I5" s="5" t="n">
+        <v>305.158</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="1" t="inlineStr">
+        <is>
+          <t>Bays Tall</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="n">
+        <v>2</v>
+      </c>
+      <c r="E6" t="inlineStr">
+        <is>
+          <t>Horizontal Horizontal Screw Spline Assembly</t>
+        </is>
+      </c>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>BE9-2515</t>
+        </is>
+      </c>
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>0.08ft, 3.97ft, 3.97ft, 3.97ft</t>
+        </is>
+      </c>
+      <c r="H6" s="5" t="n">
+        <v>527</v>
+      </c>
+      <c r="I6" s="5" t="n">
+        <v>323.578</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="1" t="inlineStr">
+        <is>
+          <t>Custom Bay Widths</t>
+        </is>
+      </c>
+      <c r="B7" s="2" t="inlineStr">
+        <is>
+          <t>1.00 in, 47.67 in, 47.67 in, 47.67 in</t>
+        </is>
+      </c>
+      <c r="E7" t="inlineStr">
+        <is>
+          <t>Horizontal Head</t>
+        </is>
+      </c>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>BE9-2514</t>
+        </is>
+      </c>
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>0.08ft, 3.97ft, 3.97ft, 3.97ft</t>
+        </is>
+      </c>
+      <c r="H7" s="5" t="n">
+        <v>444</v>
+      </c>
+      <c r="I7" s="5" t="n">
+        <v>272.616</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="1" t="inlineStr">
+        <is>
+          <t>Custom Bay Heights</t>
+        </is>
+      </c>
+      <c r="B8" s="2" t="inlineStr">
+        <is>
+          <t>2.00 in, 94.00 in</t>
+        </is>
+      </c>
+      <c r="E8" t="inlineStr">
+        <is>
+          <t>Thermal Sill Flashing</t>
+        </is>
+      </c>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>BE9-2578</t>
+        </is>
+      </c>
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>12ft</t>
+        </is>
+      </c>
+      <c r="H8" s="5" t="n">
+        <v>264</v>
+      </c>
+      <c r="I8" s="5" t="n">
+        <v>162.096</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="1" t="inlineStr">
+        <is>
+          <t>Opening Width</t>
+        </is>
+      </c>
+      <c r="B9" s="2" t="inlineStr">
+        <is>
+          <t>144.00 in</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>Horizontal Glass Stop (Use with BE9-2514, BE9-2515, BE9-2517)</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>E9-2519</t>
+        </is>
+      </c>
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>0.08ft, 3.97ft, 3.97ft, 3.97ft, 0.08ft, 3.97ft, 3.97ft, 3.97ft</t>
+        </is>
+      </c>
+      <c r="H9" s="5" t="n">
+        <v>170.1</v>
+      </c>
+      <c r="I9" s="5" t="n">
+        <v>104.4414</v>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="1" t="inlineStr">
+        <is>
+          <t>Opening Height</t>
+        </is>
+      </c>
+      <c r="B10" s="2" t="inlineStr">
+        <is>
+          <t>96.00 in</t>
+        </is>
+      </c>
+      <c r="E10" s="7" t="n"/>
+      <c r="F10" s="7" t="n"/>
+      <c r="G10" s="8" t="inlineStr">
+        <is>
+          <t>Total Profile Cost</t>
+        </is>
+      </c>
+      <c r="H10" s="9" t="n">
+        <v>2890.1</v>
+      </c>
+      <c r="I10" s="9" t="n">
+        <v>1774.5214</v>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="1" t="inlineStr">
+        <is>
+          <t>Sq Ft per Type</t>
+        </is>
+      </c>
+      <c r="B11" s="2" t="inlineStr">
+        <is>
+          <t>96.00 sqft</t>
+        </is>
+      </c>
+      <c r="E11" s="3" t="inlineStr">
+        <is>
+          <t>ACCESSORIES</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
+        <is>
+          <t>Total Sq Ft</t>
+        </is>
+      </c>
+      <c r="B12" s="2" t="inlineStr">
+        <is>
+          <t>96.00 sqft</t>
+        </is>
+      </c>
+      <c r="E12" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F12" s="4" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G12" s="4" t="inlineStr">
+        <is>
+          <t>Total Quantity Required</t>
+        </is>
+      </c>
+      <c r="H12" s="4" t="inlineStr">
+        <is>
+          <t>Total List Cost</t>
+        </is>
+      </c>
+      <c r="I12" s="4" t="inlineStr">
+        <is>
+          <t>Discounted Total List Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
+        <is>
+          <t>Perimeter Ft</t>
+        </is>
+      </c>
+      <c r="B13" s="2" t="inlineStr">
+        <is>
+          <t>40.00 ft</t>
+        </is>
+      </c>
+      <c r="E13" t="inlineStr">
+        <is>
+          <t>End Dam For Sill Flashing</t>
+        </is>
+      </c>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>E1-0199</t>
+        </is>
+      </c>
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>2.00 pcs</t>
+        </is>
+      </c>
+      <c r="H13" s="5" t="n">
+        <v>64.8</v>
+      </c>
+      <c r="I13" s="5" t="n">
+        <v>39.7872</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="1" t="inlineStr">
+        <is>
+          <t>Total Perimeter Ft</t>
+        </is>
+      </c>
+      <c r="B14" s="2" t="inlineStr">
+        <is>
+          <t>40.00 ft</t>
+        </is>
+      </c>
+      <c r="E14" t="inlineStr">
+        <is>
+          <t>Water Deflector</t>
+        </is>
+      </c>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>E2-0047</t>
+        </is>
+      </c>
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="H14" s="5" t="n">
+        <v>119</v>
+      </c>
+      <c r="I14" s="5" t="n">
+        <v>73.066</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="1" t="inlineStr">
+        <is>
+          <t>Doors</t>
+        </is>
+      </c>
+      <c r="B15" s="2" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
+      </c>
+      <c r="E15" t="inlineStr">
+        <is>
+          <t>#12 x 1-1/4” PHSMS Type AB, Zinc Plated Steel, For Screw Spline Attachment</t>
+        </is>
+      </c>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>PC-1220</t>
+        </is>
+      </c>
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>56.00 pcs</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="n">
+        <v>18.3</v>
+      </c>
+      <c r="I15" s="5" t="n">
+        <v>11.2362</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>#10-24 x 3/8” PHMS, Stainless Steel, For Attachment of Sill to Sill Flashing</t>
+        </is>
+      </c>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>PM-1006-SS</t>
+        </is>
+      </c>
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>12.00 pcs</t>
+        </is>
+      </c>
+      <c r="H16" s="5" t="n">
+        <v>46.65</v>
+      </c>
+      <c r="I16" s="5" t="n">
+        <v>28.6431</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="A17" s="3" t="inlineStr">
+        <is>
+          <t>Bay Distribution Diagram</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>*Note - C/L Dimensions</t>
+        </is>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>#12 x 3/4” UFHSMS Type A, Zinc Plated Steel For End Dam Attachment</t>
+        </is>
+      </c>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>UA-1212</t>
+        </is>
+      </c>
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="n">
+        <v>48.6</v>
+      </c>
+      <c r="I17" s="5" t="n">
+        <v>29.8404</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>Setting Block Chair Use with E2-0177 Setting Block at Sill</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>E1-2530</t>
+        </is>
+      </c>
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="H18" s="5" t="n">
+        <v>36</v>
+      </c>
+      <c r="I18" s="5" t="n">
+        <v>22.104</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="E19" t="inlineStr">
+        <is>
+          <t>Side Block For Intermediate Vertical Shallow Pocket</t>
+        </is>
+      </c>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>E2-0166</t>
+        </is>
+      </c>
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>6.00 pcs</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="n">
+        <v>76.95</v>
+      </c>
+      <c r="I19" s="5" t="n">
+        <v>47.2473</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="E20" t="inlineStr">
+        <is>
+          <t>Setting Block For Sill</t>
+        </is>
+      </c>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>E2-0177</t>
+        </is>
+      </c>
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="H20" s="5" t="n">
+        <v>76.95</v>
+      </c>
+      <c r="I20" s="5" t="n">
+        <v>47.2473</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="E21" t="inlineStr">
+        <is>
+          <t>1-1/8” “W” Side Block For Jamb</t>
+        </is>
+      </c>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>E2-0545</t>
+        </is>
+      </c>
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>4.00 pcs</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="n">
+        <v>147</v>
+      </c>
+      <c r="I21" s="5" t="n">
+        <v>90.258</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="E22" t="inlineStr">
+        <is>
+          <t>1/2” “W” Side Block For Intermediate Vertical Deep Pocket</t>
+        </is>
+      </c>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>E2-0154</t>
+        </is>
+      </c>
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>6.00 pcs</t>
+        </is>
+      </c>
+      <c r="H22" s="5" t="n">
+        <v>56.7</v>
+      </c>
+      <c r="I22" s="5" t="n">
+        <v>34.8138</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="E23" t="inlineStr">
+        <is>
+          <t>Setting Block For Intermediate Horizontal</t>
+        </is>
+      </c>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>E2-0611</t>
+        </is>
+      </c>
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>8.00 pcs</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="n">
+        <v>95.25</v>
+      </c>
+      <c r="I23" s="5" t="n">
+        <v>58.4835</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="E24" s="7" t="n"/>
+      <c r="F24" s="7" t="n"/>
+      <c r="G24" s="8" t="inlineStr">
+        <is>
+          <t>Total Accessory Cost</t>
+        </is>
+      </c>
+      <c r="H24" s="9" t="n">
+        <v>786.2</v>
+      </c>
+      <c r="I24" s="9" t="n">
+        <v>482.7268</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="E25" s="3" t="inlineStr">
+        <is>
+          <t>GASKETS</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="E26" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F26" s="4" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G26" s="4" t="inlineStr">
+        <is>
+          <t>Total Quantity Required</t>
+        </is>
+      </c>
+      <c r="H26" s="4" t="inlineStr">
+        <is>
+          <t>Total List Cost</t>
+        </is>
+      </c>
+      <c r="I26" s="4" t="inlineStr">
+        <is>
+          <t>Discounted Total List Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Glazing Gasket For 1” Glazing</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>E2-0052</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>224.00 ft</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="n">
+        <v>405</v>
+      </c>
+      <c r="I27" s="5" t="n">
+        <v>248.67</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="E28" s="7" t="n"/>
+      <c r="F28" s="7" t="n"/>
+      <c r="G28" s="8" t="inlineStr">
+        <is>
+          <t>Total Gasket Cost</t>
+        </is>
+      </c>
+      <c r="H28" s="9" t="n">
+        <v>405</v>
+      </c>
+      <c r="I28" s="9" t="n">
+        <v>248.67</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="E29" s="3" t="inlineStr">
+        <is>
+          <t>GLASS</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="E30" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F30" s="4" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G30" s="4" t="inlineStr">
+        <is>
+          <t>Total Quantity Required</t>
+        </is>
+      </c>
+      <c r="H30" s="4" t="inlineStr">
+        <is>
+          <t>Total List Cost</t>
+        </is>
+      </c>
+      <c r="I30" s="4" t="inlineStr">
+        <is>
+          <t>Discounted Total List Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>Glass Area (Adjusted)</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>83.75 sqft</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="n">
+        <v>879.375</v>
+      </c>
+      <c r="I31" s="5" t="n">
+        <v>879.375</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="E32" s="7" t="n"/>
+      <c r="F32" s="7" t="n"/>
+      <c r="G32" s="8" t="inlineStr">
+        <is>
+          <t>Total Glass Cost</t>
+        </is>
+      </c>
+      <c r="H32" s="9" t="n">
+        <v>879.375</v>
+      </c>
+      <c r="I32" s="9" t="n">
+        <v>879.375</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="E33" s="3" t="inlineStr">
+        <is>
+          <t>FABRICATION</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="E34" s="4" t="inlineStr">
+        <is>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="F34" s="4" t="inlineStr">
+        <is>
+          <t>Part Number</t>
+        </is>
+      </c>
+      <c r="G34" s="4" t="inlineStr">
+        <is>
+          <t>Total Quantity Required</t>
+        </is>
+      </c>
+      <c r="H34" s="4" t="inlineStr">
+        <is>
+          <t>Total List Cost</t>
+        </is>
+      </c>
+      <c r="I34" s="4" t="inlineStr">
+        <is>
+          <t>Discounted Total List Cost</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>Joints Fabrication Labor</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>N/A</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>24.00 joints</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="n">
+        <v>360</v>
+      </c>
+      <c r="I35" s="5" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="36">
+      <c r="E36" s="7" t="n"/>
+      <c r="F36" s="7" t="n"/>
+      <c r="G36" s="8" t="inlineStr">
+        <is>
+          <t>Total Fabrication Cost</t>
+        </is>
+      </c>
+      <c r="H36" s="9" t="n">
+        <v>360</v>
+      </c>
+      <c r="I36" s="9" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr"/>
+    </row>
+    <row r="38">
+      <c r="G38" s="4" t="inlineStr">
+        <is>
+          <t>COST/ELEVATION</t>
+        </is>
+      </c>
+      <c r="I38" s="4" t="inlineStr">
+        <is>
+          <t>TOTAL ELEVATION COST</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>PROFILE COSTS</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="n">
+        <v>1774.5214</v>
+      </c>
+    </row>
+    <row r="40">
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>ACCESSORY COSTS</t>
+        </is>
+      </c>
+      <c r="I40" s="5" t="n">
+        <v>482.7268</v>
+      </c>
+    </row>
+    <row r="41">
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>GASKET COSTS</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="n">
+        <v>248.67</v>
+      </c>
+    </row>
+    <row r="42">
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>GLASS COSTS</t>
+        </is>
+      </c>
+      <c r="I42" s="5" t="n">
+        <v>879.375</v>
+      </c>
+    </row>
+    <row r="43">
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>FABRICATION COSTS</t>
+        </is>
+      </c>
+      <c r="I43" s="5" t="n">
+        <v>360</v>
+      </c>
+    </row>
+    <row r="44">
+      <c r="G44" s="11" t="inlineStr">
+        <is>
+          <t>1 TOTAL COSTS</t>
+        </is>
+      </c>
+      <c r="I44" s="12" t="n">
+        <v>3745.2932</v>
+      </c>
+    </row>
+    <row r="45">
+      <c r="G45" s="13" t="inlineStr">
+        <is>
+          <t>*Note - Elevation costs based on discounted material costs</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:K45"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="26" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
     <col width="2" customWidth="1" min="3" max="3"/>
     <col width="2" customWidth="1" min="4" max="4"/>
@@ -728,7 +1751,7 @@
       </c>
       <c r="B3" s="2" t="inlineStr">
         <is>
-          <t>1</t>
+          <t>1 (Copy)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
@@ -1608,7 +2631,7 @@
     <row r="44">
       <c r="G44" s="11" t="inlineStr">
         <is>
-          <t>1 TOTAL COSTS</t>
+          <t>1 (Copy) TOTAL COSTS</t>
         </is>
       </c>
       <c r="I44" s="12" t="n">
@@ -1628,7 +2651,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1721,37 +2744,37 @@
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>0.25 ft</t>
+          <t>28.25 ft</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>1 (24ft per)</t>
+          <t>2 (24ft per)</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>0ft x3</t>
+          <t>8ft x2, 4ft x3, 0ft x4</t>
         </is>
       </c>
       <c r="F3" s="5" t="n">
-        <v>419</v>
+        <v>838</v>
       </c>
       <c r="G3" s="5" t="n">
-        <v>257.266</v>
+        <v>514.532</v>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>23.75ft x1</t>
+          <t>19.69ft x1, 0.06ft x1</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>98.96%</t>
+          <t>41.15%</t>
         </is>
       </c>
       <c r="J3" s="5" t="n">
-        <v>254.5861458333333</v>
+        <v>211.7083898381944</v>
       </c>
     </row>
     <row r="4">
@@ -1767,24 +2790,24 @@
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
         <is>
-          <t>0 (24ft per)</t>
+          <t>1 (24ft per)</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>24ft x1, 8ft x3</t>
         </is>
       </c>
       <c r="F4" s="5" t="n">
-        <v>0</v>
+        <v>300</v>
       </c>
       <c r="G4" s="5" t="n">
-        <v>0</v>
+        <v>184.2</v>
       </c>
       <c r="H4" t="inlineStr">
         <is>
@@ -1813,24 +2836,24 @@
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>24.00 ft</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>0 (24ft per)</t>
+          <t>1 (24ft per)</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>0.00 ft</t>
+          <t>24ft x1, 8ft x3</t>
         </is>
       </c>
       <c r="F5" s="5" t="n">
-        <v>0</v>
+        <v>994</v>
       </c>
       <c r="G5" s="5" t="n">
-        <v>0</v>
+        <v>610.316</v>
       </c>
       <c r="H5" t="inlineStr">
         <is>
@@ -1859,7 +2882,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>12.08 ft</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
@@ -1869,7 +2892,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>0ft</t>
+          <t>4ft x3, 0ft x2</t>
         </is>
       </c>
       <c r="F6" s="5" t="n">
@@ -1880,16 +2903,16 @@
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>23.92ft x1</t>
+          <t>11.92ft x1</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>99.65%</t>
+          <t>49.65%</t>
         </is>
       </c>
       <c r="J6" s="5" t="n">
-        <v>322.4544652777778</v>
+        <v>160.6653529243055</v>
       </c>
     </row>
     <row r="7">
@@ -1905,7 +2928,7 @@
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>12.08 ft</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
@@ -1915,7 +2938,7 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>0ft</t>
+          <t>4ft x3, 0ft x2</t>
         </is>
       </c>
       <c r="F7" s="5" t="n">
@@ -1926,16 +2949,16 @@
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>23.92ft x1</t>
+          <t>11.92ft x1</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>99.65%</t>
+          <t>49.65%</t>
         </is>
       </c>
       <c r="J7" s="5" t="n">
-        <v>271.6694166666667</v>
+        <v>135.3613220083333</v>
       </c>
     </row>
     <row r="8">
@@ -1951,7 +2974,7 @@
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>12.08 ft</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
@@ -1961,7 +2984,7 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>0ft</t>
+          <t>12ft x1, 0ft x1</t>
         </is>
       </c>
       <c r="F8" s="5" t="n">
@@ -1972,16 +2995,16 @@
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>23.92ft x1</t>
+          <t>11.92ft x1</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>99.65%</t>
+          <t>49.65%</t>
         </is>
       </c>
       <c r="J8" s="5" t="n">
-        <v>161.5331666666667</v>
+        <v>80.48516666666666</v>
       </c>
     </row>
     <row r="9">
@@ -1997,37 +3020,37 @@
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>0.08 ft</t>
+          <t>24.08 ft</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>1 (24ft per)</t>
+          <t>2 (24ft per)</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>0ft</t>
+          <t>4ft x6, 0ft x3</t>
         </is>
       </c>
       <c r="F9" s="5" t="n">
-        <v>85.05</v>
+        <v>170.1</v>
       </c>
       <c r="G9" s="5" t="n">
-        <v>52.2207</v>
+        <v>104.4414</v>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>23.92ft x1</t>
+          <t>23.83ft x1, 0.08ft x1</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>99.65%</t>
+          <t>49.83%</t>
         </is>
       </c>
       <c r="J9" s="5" t="n">
-        <v>52.039378125</v>
+        <v>52.039341860625</v>
       </c>
     </row>
     <row r="10">
@@ -2041,15 +3064,15 @@
         </is>
       </c>
       <c r="F10" s="9" t="n">
-        <v>1739.05</v>
+        <v>3537.1</v>
       </c>
       <c r="G10" s="9" t="n">
-        <v>1067.7767</v>
+        <v>2171.7794</v>
       </c>
       <c r="H10" s="7" t="n"/>
       <c r="I10" s="7" t="n"/>
       <c r="J10" s="9" t="n">
-        <v>1062.282572569445</v>
+        <v>640.2595732981248</v>
       </c>
     </row>
     <row r="11">
@@ -2124,7 +3147,7 @@
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>4.00 pcs</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
@@ -2145,16 +3168,16 @@
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>18.00 pcs</t>
+          <t>16.00 pcs</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>90.00%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="J13" s="5" t="n">
-        <v>35.80848</v>
+        <v>31.82976</v>
       </c>
     </row>
     <row r="14">
@@ -2170,7 +3193,7 @@
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>10.00 pcs</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -2191,16 +3214,16 @@
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>40.00 pcs</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>96.00%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="J14" s="5" t="n">
-        <v>70.14336</v>
+        <v>58.45279999999999</v>
       </c>
     </row>
     <row r="15">
@@ -2216,7 +3239,7 @@
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>8.00 pcs</t>
+          <t>64.00 pcs</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -2237,16 +3260,16 @@
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>92.00 pcs</t>
+          <t>36.00 pcs</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>92.00%</t>
+          <t>36.00%</t>
         </is>
       </c>
       <c r="J15" s="5" t="n">
-        <v>10.337304</v>
+        <v>4.045032</v>
       </c>
     </row>
     <row r="16">
@@ -2262,7 +3285,7 @@
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>3.00 pcs</t>
+          <t>15.00 pcs</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
@@ -2283,16 +3306,16 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>97.00 pcs</t>
+          <t>85.00 pcs</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>97.00%</t>
+          <t>85.00%</t>
         </is>
       </c>
       <c r="J16" s="5" t="n">
-        <v>27.783807</v>
+        <v>24.346635</v>
       </c>
     </row>
     <row r="17">
@@ -2308,7 +3331,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>4.00 pcs</t>
+          <t>8.00 pcs</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -2329,16 +3352,16 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>96.00 pcs</t>
+          <t>92.00 pcs</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>96.00%</t>
+          <t>92.00%</t>
         </is>
       </c>
       <c r="J17" s="5" t="n">
-        <v>28.646784</v>
+        <v>27.453168</v>
       </c>
     </row>
     <row r="18">
@@ -2354,7 +3377,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>10.00 pcs</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
@@ -2364,14 +3387,14 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>2 orders</t>
+          <t>10 orders</t>
         </is>
       </c>
       <c r="F18" s="5" t="n">
-        <v>9</v>
+        <v>45</v>
       </c>
       <c r="G18" s="5" t="n">
-        <v>5.526</v>
+        <v>27.63</v>
       </c>
       <c r="H18" t="inlineStr">
         <is>
@@ -2400,7 +3423,7 @@
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
@@ -2410,27 +3433,27 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>0 orders</t>
+          <t>1 order</t>
         </is>
       </c>
       <c r="F19" s="5" t="n">
-        <v>0</v>
+        <v>76.95</v>
       </c>
       <c r="G19" s="5" t="n">
-        <v>0</v>
+        <v>47.2473</v>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>88.00%</t>
         </is>
       </c>
       <c r="J19" s="5" t="n">
-        <v>0</v>
+        <v>41.57762400000001</v>
       </c>
     </row>
     <row r="20">
@@ -2446,7 +3469,7 @@
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>10.00 pcs</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -2467,16 +3490,16 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>40.00 pcs</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>96.00%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="J20" s="5" t="n">
-        <v>45.35740800000001</v>
+        <v>37.79784</v>
       </c>
     </row>
     <row r="21">
@@ -2492,7 +3515,7 @@
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
@@ -2513,16 +3536,16 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>96.00%</t>
+          <t>88.00%</t>
         </is>
       </c>
       <c r="J21" s="5" t="n">
-        <v>86.64768000000001</v>
+        <v>79.42703999999999</v>
       </c>
     </row>
     <row r="22">
@@ -2538,7 +3561,7 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>6.00 pcs</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -2548,27 +3571,27 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>0 orders</t>
+          <t>1 order</t>
         </is>
       </c>
       <c r="F22" s="5" t="n">
-        <v>0</v>
+        <v>56.7</v>
       </c>
       <c r="G22" s="5" t="n">
-        <v>0</v>
+        <v>34.8138</v>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>0.00 pcs</t>
+          <t>44.00 pcs</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>0.00%</t>
+          <t>88.00%</t>
         </is>
       </c>
       <c r="J22" s="5" t="n">
-        <v>0</v>
+        <v>30.63614400000001</v>
       </c>
     </row>
     <row r="23">
@@ -2584,7 +3607,7 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>2.00 pcs</t>
+          <t>10.00 pcs</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
@@ -2605,16 +3628,16 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>48.00 pcs</t>
+          <t>40.00 pcs</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>96.00%</t>
+          <t>80.00%</t>
         </is>
       </c>
       <c r="J23" s="5" t="n">
-        <v>56.14416</v>
+        <v>46.7868</v>
       </c>
     </row>
     <row r="24">
@@ -2628,15 +3651,15 @@
         </is>
       </c>
       <c r="F24" s="9" t="n">
-        <v>625.55</v>
+        <v>795.2</v>
       </c>
       <c r="G24" s="9" t="n">
-        <v>384.0877</v>
+        <v>488.2528</v>
       </c>
       <c r="H24" s="7" t="n"/>
       <c r="I24" s="7" t="n"/>
       <c r="J24" s="9" t="n">
-        <v>360.868983</v>
+        <v>382.352843</v>
       </c>
     </row>
     <row r="25">
@@ -2711,7 +3734,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>0.67 ft</t>
+          <t>224.67 ft</t>
         </is>
       </c>
       <c r="D27" t="inlineStr">
@@ -2721,7 +3744,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>1ft</t>
+          <t>224ft x1, 1ft x1</t>
         </is>
       </c>
       <c r="F27" s="5" t="n">
@@ -2732,16 +3755,16 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>499.33ft x1</t>
+          <t>275.33ft x1</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>99.87%</t>
+          <t>55.07%</t>
         </is>
       </c>
       <c r="J27" s="5" t="n">
-        <v>248.33844</v>
+        <v>136.93428</v>
       </c>
     </row>
     <row r="28">
@@ -2763,7 +3786,7 @@
       <c r="H28" s="7" t="n"/>
       <c r="I28" s="7" t="n"/>
       <c r="J28" s="9" t="n">
-        <v>248.33844</v>
+        <v>136.93428</v>
       </c>
     </row>
     <row r="29">
@@ -2848,14 +3871,14 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>0.06 sqft</t>
+          <t>83.81 sqft</t>
         </is>
       </c>
       <c r="F31" s="5" t="n">
-        <v>0.65625</v>
+        <v>880.03125</v>
       </c>
       <c r="G31" s="5" t="n">
-        <v>0.65625</v>
+        <v>880.03125</v>
       </c>
       <c r="H31" t="inlineStr">
         <is>
@@ -2882,10 +3905,10 @@
         </is>
       </c>
       <c r="F32" s="9" t="n">
-        <v>0.65625</v>
+        <v>880.03125</v>
       </c>
       <c r="G32" s="9" t="n">
-        <v>0.65625</v>
+        <v>880.03125</v>
       </c>
       <c r="H32" s="7" t="n"/>
       <c r="I32" s="7" t="n"/>
@@ -2975,14 +3998,14 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>4.00 joints</t>
+          <t>28.00 joints</t>
         </is>
       </c>
       <c r="F35" s="5" t="n">
-        <v>60</v>
+        <v>420</v>
       </c>
       <c r="G35" s="5" t="n">
-        <v>60</v>
+        <v>420</v>
       </c>
       <c r="H35" t="inlineStr">
         <is>
@@ -3009,10 +4032,10 @@
         </is>
       </c>
       <c r="F36" s="9" t="n">
-        <v>60</v>
+        <v>420</v>
       </c>
       <c r="G36" s="9" t="n">
-        <v>60</v>
+        <v>420</v>
       </c>
       <c r="H36" s="7" t="n"/>
       <c r="I36" s="7" t="n"/>
@@ -3036,7 +4059,7 @@
         </is>
       </c>
       <c r="C38" s="18" t="n">
-        <v>2830.25625</v>
+        <v>6037.33125</v>
       </c>
     </row>
     <row r="39">
@@ -3046,7 +4069,7 @@
         </is>
       </c>
       <c r="C39" s="20" t="n">
-        <v>1761.19065</v>
+        <v>4208.73345</v>
       </c>
     </row>
     <row r="40">
@@ -3056,7 +4079,7 @@
         </is>
       </c>
       <c r="C40" s="18" t="n">
-        <v>1671.489995569445</v>
+        <v>1159.546696298125</v>
       </c>
     </row>
     <row r="41">
@@ -3068,7 +4091,7 @@
       <c r="B41" s="22" t="n"/>
       <c r="C41" s="23" t="inlineStr">
         <is>
-          <t>94.91%</t>
+          <t>27.55%</t>
         </is>
       </c>
     </row>
@@ -3145,7 +4168,7 @@
       </c>
       <c r="B49" s="39" t="n"/>
       <c r="C49" s="40" t="n">
-        <v>1761.19065</v>
+        <v>4208.73345</v>
       </c>
     </row>
     <row r="50">
@@ -3176,7 +4199,7 @@
       </c>
       <c r="B52" s="42" t="n"/>
       <c r="C52" s="43" t="n">
-        <v>1761.19065</v>
+        <v>4208.73345</v>
       </c>
     </row>
   </sheetData>

</xml_diff>